<commit_message>
new cell surface data and chimp cell number
</commit_message>
<xml_diff>
--- a/Young_etal_2013/Young_etal_2013.xlsx
+++ b/Young_etal_2013/Young_etal_2013.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/Young_etal_2013/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{87A38D43-FB4B-164F-A4C4-1EF284968B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0ED6C3B-6742-9A40-A29D-6BF541F2ACAD}"/>
+  <xr:revisionPtr revIDLastSave="237" documentId="8_{87A38D43-FB4B-164F-A4C4-1EF284968B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8980D19-2394-E748-B191-5B443867FCE5}"/>
   <bookViews>
-    <workbookView xWindow="37840" yWindow="1420" windowWidth="29160" windowHeight="16420" activeTab="1" xr2:uid="{F73B9AFC-2043-5248-B344-8270F8690E1E}"/>
+    <workbookView xWindow="52660" yWindow="280" windowWidth="29160" windowHeight="16420" activeTab="1" xr2:uid="{F73B9AFC-2043-5248-B344-8270F8690E1E}"/>
   </bookViews>
   <sheets>
     <sheet name="published Table 1" sheetId="1" r:id="rId1"/>
@@ -2101,14 +2101,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2367,39 +2365,56 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57F5FEC8-D08D-4145-ABC7-B3A613D5D4C0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C8F1AC2-6B39-4F5D-BF4A-736165E42A2F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9574DCAA-0DC8-4FD9-B486-4FC4712ACA66}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9574DCAA-0DC8-4FD9-B486-4FC4712ACA66}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C8F1AC2-6B39-4F5D-BF4A-736165E42A2F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57F5FEC8-D08D-4145-ABC7-B3A613D5D4C0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>